<commit_message>
Pembaharuan 20 juli 2026
</commit_message>
<xml_diff>
--- a/Contoh Template File/Nota.xlsx
+++ b/Contoh Template File/Nota.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Pekerjaan\Contoh Template File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA598FD-6698-4468-BED3-3DFAB0EDC3BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8186D44A-6A80-4C1E-BE3E-5F7F3FF968D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>NO.</t>
   </si>
@@ -137,6 +137,9 @@
       </rPr>
       <t>Juli 2026</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">No : </t>
   </si>
 </sst>
 </file>
@@ -468,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -556,6 +559,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -599,10 +605,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -635,7 +644,7 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>2738436</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>63962</xdr:rowOff>
+      <xdr:rowOff>75868</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -677,13 +686,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>154781</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>23812</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>2320131</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>79851</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1018,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B5:N37"/>
+  <dimension ref="B5:N38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" customWidth="1"/>
@@ -1034,47 +1043,47 @@
     <row r="5" spans="2:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="2:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
     </row>
     <row r="8" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
     </row>
     <row r="9" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
     </row>
     <row r="10" spans="2:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
     </row>
     <row r="11" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C11" s="41" t="s">
+      <c r="C11" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
     </row>
     <row r="12" spans="2:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F12" s="17"/>
@@ -1084,10 +1093,10 @@
       <c r="B13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="49" t="s">
+      <c r="F13" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="49"/>
+      <c r="G13" s="50"/>
       <c r="N13" s="6" t="s">
         <v>16</v>
       </c>
@@ -1097,56 +1106,58 @@
       <c r="C14" s="51"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="50" t="s">
+      <c r="F14" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="50"/>
-    </row>
-    <row r="15" spans="2:14" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="9"/>
-      <c r="D15" s="10"/>
-    </row>
-    <row r="16" spans="2:14" s="1" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
+      <c r="G14" s="52"/>
+    </row>
+    <row r="15" spans="2:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="53"/>
+    </row>
+    <row r="16" spans="2:14" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="9"/>
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" spans="2:7" s="1" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D17" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E17" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F17" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G17" s="19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="8"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="28"/>
-    </row>
-    <row r="18" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="29"/>
+    <row r="18" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="8"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="27"/>
       <c r="G18" s="28"/>
     </row>
     <row r="19" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="33"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="E19" s="12"/>
       <c r="F19" s="29"/>
       <c r="G19" s="28"/>
     </row>
@@ -1159,11 +1170,11 @@
       <c r="G20" s="28"/>
     </row>
     <row r="21" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="5"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="30"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="29"/>
       <c r="G21" s="28"/>
     </row>
     <row r="22" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1206,92 +1217,101 @@
       <c r="F26" s="30"/>
       <c r="G26" s="28"/>
     </row>
-    <row r="27" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
+      <c r="C27" s="34"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
       <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-    </row>
-    <row r="28" spans="2:7" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="44" t="s">
+      <c r="G27" s="28"/>
+    </row>
+    <row r="28" spans="2:7" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+    </row>
+    <row r="29" spans="2:7" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="31">
-        <f>SUM(G17:G27)</f>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="31">
+        <f>SUM(G18:G28)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="21"/>
-    </row>
-    <row r="31" spans="2:7" s="23" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B31" s="47" t="s">
+    <row r="30" spans="2:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="21"/>
+    </row>
+    <row r="32" spans="2:7" s="23" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B32" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="47"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="48" t="s">
+      <c r="C32" s="48"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="G31" s="48"/>
-    </row>
-    <row r="35" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B35" s="38"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="38"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="42" t="s">
+      <c r="G32" s="49"/>
+    </row>
+    <row r="36" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B37" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="C36" s="43"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="25"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="39" t="s">
+      <c r="C37" s="44"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="44"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="25"/>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="40"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="25"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="C7:G8"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B38:G38"/>
     <mergeCell ref="C11:G11"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="F32:G32"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="B14:C14"/>
+    <mergeCell ref="F15:G15"/>
   </mergeCells>
   <pageMargins left="0.47" right="0.23622047244094491" top="7.874015748031496E-2" bottom="0.74803149606299213" header="0.59055118110236227" footer="0.31496062992125984"/>
   <pageSetup paperSize="5" scale="83" orientation="portrait" horizontalDpi="4294967294" verticalDpi="300" r:id="rId1"/>

</xml_diff>